<commit_message>
Acronym strating with factor initial
</commit_message>
<xml_diff>
--- a/Reproduce6 - AnalysisBySystem/ItemsCodeSig.xlsx
+++ b/Reproduce6 - AnalysisBySystem/ItemsCodeSig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eliane\My_codes\GitSuppMaterial\Phase 3 - Scale Validation\Reproduce6 - AnalysisBySystem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C9D446B-C4E2-4826-89BE-7B9CCD0F709B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60395832-EEF3-4B1F-AB80-D4F4FBE2F3CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1A7D0A9D-1F3A-4C75-B9CF-B4BABEB84DCD}"/>
   </bookViews>
@@ -39,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
-  <si>
-    <t>visSimpleUnderstand</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="42">
   <si>
     <t>P089 The visual representations I saw were simple to understand</t>
   </si>
@@ -56,9 +53,6 @@
     <t>P022A</t>
   </si>
   <si>
-    <t>trialError</t>
-  </si>
-  <si>
     <t>P067.I.could.safely.engage.in.a.trial.and.error.analysis.processï</t>
   </si>
   <si>
@@ -77,18 +71,12 @@
     <t>P064</t>
   </si>
   <si>
-    <t>visAppropriate</t>
-  </si>
-  <si>
     <t>P098 I found the visual representations provided by the system were appropriate</t>
   </si>
   <si>
     <t>P098</t>
   </si>
   <si>
-    <t>visFaithful</t>
-  </si>
-  <si>
     <t>P106 The visualizations I saw seemed to represent the data faithfully</t>
   </si>
   <si>
@@ -131,31 +119,52 @@
     <t>P301</t>
   </si>
   <si>
-    <t>sysSimpleUnderstand</t>
-  </si>
-  <si>
-    <t>sysEnjoy</t>
-  </si>
-  <si>
-    <t>sysUseful</t>
-  </si>
-  <si>
-    <t>analysisConfigure</t>
-  </si>
-  <si>
-    <t>sysEasyStart</t>
-  </si>
-  <si>
-    <t>sysRetrieveInfo</t>
-  </si>
-  <si>
-    <t>sysThinkDeep</t>
-  </si>
-  <si>
-    <t>visRemember</t>
-  </si>
-  <si>
-    <t>taskComplete</t>
+    <t>Vis</t>
+  </si>
+  <si>
+    <t>Intuitiveness</t>
+  </si>
+  <si>
+    <t>Cognitive</t>
+  </si>
+  <si>
+    <t>CogSysThinkDeep</t>
+  </si>
+  <si>
+    <t>CogTaskComplete</t>
+  </si>
+  <si>
+    <t>CogSysEnjoy</t>
+  </si>
+  <si>
+    <t>CogSysUseful</t>
+  </si>
+  <si>
+    <t>IntSysEasyStart</t>
+  </si>
+  <si>
+    <t>IntAnalysisConfigure</t>
+  </si>
+  <si>
+    <t>IntSysSimpleUnderstand</t>
+  </si>
+  <si>
+    <t>VisSimpleUnderstand</t>
+  </si>
+  <si>
+    <t>VisRemember</t>
+  </si>
+  <si>
+    <t>VisTrialError</t>
+  </si>
+  <si>
+    <t>VisSysRetrieveInfo</t>
+  </si>
+  <si>
+    <t>VisAppropriate</t>
+  </si>
+  <si>
+    <t>VisFaithful</t>
   </si>
 </sst>
 </file>
@@ -230,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -242,6 +251,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -578,249 +594,292 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{581BB7C1-2D9D-4890-8B44-39FA3DA72E82}">
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:S13"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="38.6328125" customWidth="1"/>
-    <col min="2" max="2" width="27.54296875" customWidth="1"/>
-    <col min="3" max="3" width="56.08984375" customWidth="1"/>
+    <col min="1" max="1" width="23.7265625" customWidth="1"/>
+    <col min="2" max="2" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="27.54296875" customWidth="1"/>
+    <col min="4" max="4" width="56.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
+    <row r="1" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" t="s">
-        <v>19</v>
+        <v>29</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="G1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="H1" t="s">
         <v>21</v>
       </c>
       <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>3</v>
+      </c>
+      <c r="K1" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R1" t="s">
+        <v>9</v>
+      </c>
+      <c r="S1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="str">
+        <f>VLOOKUP(G1, $B:$C, 2, FALSE)</f>
+        <v>IntSysEasyStart</v>
+      </c>
+      <c r="H2" t="str">
+        <f>VLOOKUP(H1, $B:$C, 2, FALSE)</f>
+        <v>IntSysSimpleUnderstand</v>
+      </c>
+      <c r="I2" t="str">
+        <f t="shared" ref="I2:S2" si="0">VLOOKUP(I1, $B:$C, 2, FALSE)</f>
+        <v>IntAnalysisConfigure</v>
+      </c>
+      <c r="J2" t="str">
+        <f t="shared" si="0"/>
+        <v>VisRemember</v>
+      </c>
+      <c r="K2" t="str">
+        <f t="shared" si="0"/>
+        <v>VisTrialError</v>
+      </c>
+      <c r="L2" t="str">
+        <f t="shared" si="0"/>
+        <v>VisSimpleUnderstand</v>
+      </c>
+      <c r="M2" t="str">
+        <f t="shared" si="0"/>
+        <v>VisSysRetrieveInfo</v>
+      </c>
+      <c r="N2" t="str">
+        <f t="shared" si="0"/>
+        <v>VisAppropriate</v>
+      </c>
+      <c r="O2" t="str">
+        <f t="shared" si="0"/>
+        <v>VisFaithful</v>
+      </c>
+      <c r="P2" t="str">
+        <f t="shared" si="0"/>
+        <v>CogTaskComplete</v>
+      </c>
+      <c r="Q2" t="str">
+        <f t="shared" si="0"/>
+        <v>CogSysEnjoy</v>
+      </c>
+      <c r="R2" t="str">
+        <f t="shared" si="0"/>
+        <v>CogSysThinkDeep</v>
+      </c>
+      <c r="S2" t="str">
+        <f t="shared" si="0"/>
+        <v>CogSysUseful</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="J1" t="s">
+    </row>
+    <row r="11" spans="1:19" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
-        <v>2</v>
-      </c>
-      <c r="L1" t="s">
-        <v>9</v>
-      </c>
-      <c r="M1" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" t="s">
-        <v>17</v>
-      </c>
-      <c r="O1" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" t="s">
+      <c r="C11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="R1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" t="str">
-        <f>VLOOKUP(F1, $A:$B, 2, FALSE)</f>
-        <v>sysEasyStart</v>
-      </c>
-      <c r="G2" t="str">
-        <f>VLOOKUP(G1, $A:$B, 2, FALSE)</f>
-        <v>sysSimpleUnderstand</v>
-      </c>
-      <c r="H2" t="str">
-        <f t="shared" ref="H2:R2" si="0">VLOOKUP(H1, $A:$B, 2, FALSE)</f>
-        <v>analysisConfigure</v>
-      </c>
-      <c r="I2" t="str">
-        <f t="shared" si="0"/>
-        <v>visRemember</v>
-      </c>
-      <c r="J2" t="str">
-        <f t="shared" si="0"/>
-        <v>trialError</v>
-      </c>
-      <c r="K2" t="str">
-        <f t="shared" si="0"/>
-        <v>visSimpleUnderstand</v>
-      </c>
-      <c r="L2" t="str">
-        <f t="shared" si="0"/>
-        <v>sysRetrieveInfo</v>
-      </c>
-      <c r="M2" t="str">
-        <f t="shared" si="0"/>
-        <v>visAppropriate</v>
-      </c>
-      <c r="N2" t="str">
-        <f t="shared" si="0"/>
-        <v>visFaithful</v>
-      </c>
-      <c r="O2" t="str">
-        <f t="shared" si="0"/>
-        <v>taskComplete</v>
-      </c>
-      <c r="P2" t="str">
-        <f t="shared" si="0"/>
-        <v>sysEnjoy</v>
-      </c>
-      <c r="Q2" t="str">
-        <f t="shared" si="0"/>
-        <v>sysThinkDeep</v>
-      </c>
-      <c r="R2" t="str">
-        <f t="shared" si="0"/>
-        <v>sysUseful</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="C12" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
+    <row r="13" spans="1:19" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>28</v>
-      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:D13">
+    <sortCondition ref="A1:A13"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>